<commit_message>
chore: handover遡及登録 - BUG-007〜013追加・ISSUE-004解決済に更新
- BUG-007: load_mesh_tile() 前行ゼロリセットバグ（2026-04-18修正済）
- BUG-008: コル検出バグ（海面境界誤検出、2026-04-19修正済）
- BUG-009: 整数オーバーフロー/SIGSEGV（5239解析で2.7億px超過、2026-04-24修正済）
- BUG-010: dem10b URL誤設定（2026-04-24修正済）
- BUG-011: dem10b座標変換バグ（格子状パターン、2026-04-25修正済）
- BUG-012: DEFAULT_SUMMITSLIST パス誤設定（2026-04-26修正済）
- BUG-013: analyze.c malloc NULL チェック漏れ（未対応/低）
- ISSUE-004: output_geojson.py 実装確認済みのため解決済に更新
- bugs_export.xlsx / issues_export.xlsx 再生成（13件/9件）

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/.claude/mgmt/bug-system/reports/bugs_export.xlsx
+++ b/.claude/mgmt/bug-system/reports/bugs_export.xlsx
@@ -45,7 +45,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -80,6 +80,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F0F0F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFE0E0"/>
       </patternFill>
     </fill>
     <fill>
@@ -119,7 +124,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -139,11 +144,14 @@
     <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -272,12 +280,12 @@
           </marker>
           <xVal>
             <numRef>
-              <f>'欠陥収束'!$A$2:$A$4</f>
+              <f>'欠陥収束'!$A$2:$A$11</f>
             </numRef>
           </xVal>
           <yVal>
             <numRef>
-              <f>'欠陥収束'!$B$2:$B$4</f>
+              <f>'欠陥収束'!$B$2:$B$11</f>
             </numRef>
           </yVal>
         </ser>
@@ -306,12 +314,12 @@
           </marker>
           <xVal>
             <numRef>
-              <f>'欠陥収束'!$A$2:$A$4</f>
+              <f>'欠陥収束'!$A$2:$A$11</f>
             </numRef>
           </xVal>
           <yVal>
             <numRef>
-              <f>'欠陥収束'!$C$2:$C$4</f>
+              <f>'欠陥収束'!$C$2:$C$11</f>
             </numRef>
           </yVal>
         </ser>
@@ -340,12 +348,12 @@
           </marker>
           <xVal>
             <numRef>
-              <f>'欠陥収束'!$A$2:$A$4</f>
+              <f>'欠陥収束'!$A$2:$A$11</f>
             </numRef>
           </xVal>
           <yVal>
             <numRef>
-              <f>'欠陥収束'!$D$2:$D$4</f>
+              <f>'欠陥収束'!$D$2:$D$11</f>
             </numRef>
           </yVal>
         </ser>
@@ -357,7 +365,7 @@
         <scaling>
           <orientation val="minMax"/>
           <max val="46139"/>
-          <min val="46137"/>
+          <min val="46130"/>
         </scaling>
         <axPos val="l"/>
         <majorGridlines/>
@@ -735,7 +743,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R7"/>
+  <dimension ref="A1:R14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1326,18 +1334,626 @@
         </is>
       </c>
     </row>
+    <row r="8" ht="40" customHeight="1">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>BUG-007</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>load_mesh_tile() 前行ゼロリセットバグ（タイル上書き破壊）</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>load_mesh_tile() でタイル書き込み後に前行を 0 リセットしていた。calloc で初期化済みのためリセット不要だが、タイルデータを上書き破壊していた致命的バグ。</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>JJ1XGO</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>COD</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>解析エンジン</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>src/mesh_analyze.c</t>
+        </is>
+      </c>
+      <c r="I8" s="6" t="inlineStr">
+        <is>
+          <t>毎回</t>
+        </is>
+      </c>
+      <c r="J8" s="7" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="K8" s="6" t="inlineStr">
+        <is>
+          <t>解決済</t>
+        </is>
+      </c>
+      <c r="L8" s="6" t="inlineStr">
+        <is>
+          <t>JJ1XGO</t>
+        </is>
+      </c>
+      <c r="M8" s="6" t="inlineStr">
+        <is>
+          <t>COD</t>
+        </is>
+      </c>
+      <c r="N8" s="6" t="inlineStr">
+        <is>
+          <t>src/mesh_analyze.c</t>
+        </is>
+      </c>
+      <c r="O8" s="6" t="inlineStr">
+        <is>
+          <t>calloc 初期化済みのため、リセットコードを削除。</t>
+        </is>
+      </c>
+      <c r="P8" s="6" t="inlineStr"/>
+      <c r="Q8" s="6" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="R8" s="6" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="40" customHeight="1">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>BUG-008</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>コル検出バグ（海面境界との接触を「コル」として誤検出）</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>Union-Find の union() 時に peak_id &lt; 0（海面コンポーネント）のチェックが抜けていた。海面境界との接触を「コル」として誤検出し、山頂の比高が過小に計算されていた。</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>JJ1XGO</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>2026-04-19</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>UT</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>解析エンジン</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>src/unionfind.c</t>
+        </is>
+      </c>
+      <c r="I9" s="6" t="inlineStr">
+        <is>
+          <t>毎回</t>
+        </is>
+      </c>
+      <c r="J9" s="7" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="K9" s="6" t="inlineStr">
+        <is>
+          <t>解決済</t>
+        </is>
+      </c>
+      <c r="L9" s="6" t="inlineStr">
+        <is>
+          <t>JJ1XGO</t>
+        </is>
+      </c>
+      <c r="M9" s="6" t="inlineStr">
+        <is>
+          <t>COD</t>
+        </is>
+      </c>
+      <c r="N9" s="6" t="inlineStr">
+        <is>
+          <t>src/unionfind.c</t>
+        </is>
+      </c>
+      <c r="O9" s="6" t="inlineStr">
+        <is>
+          <t>union 時に peak_id &lt; 0 チェックを追加して海面コンポーネントを除外。</t>
+        </is>
+      </c>
+      <c r="P9" s="6" t="inlineStr"/>
+      <c r="Q9" s="6" t="inlineStr">
+        <is>
+          <t>2026-04-19</t>
+        </is>
+      </c>
+      <c r="R9" s="6" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="40" customHeight="1">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>BUG-009</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>整数オーバーフロー/SIGSEGV（5239解析で2.7億px &gt; int32_t上限）</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>ピクセルインデックスを int32_t で管理していたため、5239 解析（70,146×38,402px = 約2.7億px）で int32_t 上限（2.1億）を超えオーバーフロー → SIGSEGV で異常終了。</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>JJ1XGO</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>解析エンジン</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>src/analyze.c, src/unionfind.h/c, src/elevation.c</t>
+        </is>
+      </c>
+      <c r="I10" s="6" t="inlineStr">
+        <is>
+          <t>毎回</t>
+        </is>
+      </c>
+      <c r="J10" s="7" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="K10" s="6" t="inlineStr">
+        <is>
+          <t>解決済</t>
+        </is>
+      </c>
+      <c r="L10" s="6" t="inlineStr">
+        <is>
+          <t>JJ1XGO</t>
+        </is>
+      </c>
+      <c r="M10" s="6" t="inlineStr">
+        <is>
+          <t>COD</t>
+        </is>
+      </c>
+      <c r="N10" s="6" t="inlineStr">
+        <is>
+          <t>src/analyze.c</t>
+        </is>
+      </c>
+      <c r="O10" s="6" t="inlineStr">
+        <is>
+          <t>ピクセルインデックスを uint32_t / size_t に変更。コミット: fb9fcfd</t>
+        </is>
+      </c>
+      <c r="P10" s="6" t="inlineStr"/>
+      <c r="Q10" s="6" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="R10" s="6" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="40" customHeight="1">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>BUG-010</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>dem10b URL誤設定（dem10b_png → dem_png）</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>prefetch_tiles.py の GSI_DEM10B_URL が dem10b_png だったが、正しいサービス名は dem_png。HTTP 404 が返り続けていたが取得漏れと区別できなかった。</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>JJ1XGO</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>prefetch</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>scripts/prefetch_tiles.py</t>
+        </is>
+      </c>
+      <c r="I11" s="6" t="inlineStr">
+        <is>
+          <t>毎回</t>
+        </is>
+      </c>
+      <c r="J11" s="5" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="K11" s="6" t="inlineStr">
+        <is>
+          <t>解決済</t>
+        </is>
+      </c>
+      <c r="L11" s="6" t="inlineStr">
+        <is>
+          <t>JJ1XGO</t>
+        </is>
+      </c>
+      <c r="M11" s="6" t="inlineStr">
+        <is>
+          <t>COD</t>
+        </is>
+      </c>
+      <c r="N11" s="6" t="inlineStr">
+        <is>
+          <t>scripts/prefetch_tiles.py</t>
+        </is>
+      </c>
+      <c r="O11" s="6" t="inlineStr">
+        <is>
+          <t>GSI_DEM10B_URL を dem_png に修正。動作確認済み（HTTP 200）。コミット: fb9fcfd</t>
+        </is>
+      </c>
+      <c r="P11" s="6" t="inlineStr"/>
+      <c r="Q11" s="6" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="R11" s="6" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="40" customHeight="1">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>BUG-011</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>dem10b座標変換バグ（terrain PNG 格子状パターンの原因）</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>elev_fill_nodata_dem10b() と elev_load_with_overlap_8dir_with_dem10() の z15→z14 ピクセル変換で * TILE_PIX（256）を使っていた。dem10b は 256×256px なのに 512×512px として扱い、z14 タイルの右半分・下半分の NODATA が補完されず terrain PNG が格子状になっていた。</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>JJ1XGO</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>解析エンジン</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>src/elevation.c</t>
+        </is>
+      </c>
+      <c r="I12" s="6" t="inlineStr">
+        <is>
+          <t>毎回</t>
+        </is>
+      </c>
+      <c r="J12" s="5" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="K12" s="6" t="inlineStr">
+        <is>
+          <t>解決済</t>
+        </is>
+      </c>
+      <c r="L12" s="6" t="inlineStr">
+        <is>
+          <t>JJ1XGO</t>
+        </is>
+      </c>
+      <c r="M12" s="6" t="inlineStr">
+        <is>
+          <t>COD</t>
+        </is>
+      </c>
+      <c r="N12" s="6" t="inlineStr">
+        <is>
+          <t>src/elevation.c</t>
+        </is>
+      </c>
+      <c r="O12" s="6" t="inlineStr">
+        <is>
+          <t>* TILE_PIX → * (TILE_PIX/2) + (px-1)/2 に修正。コミット: d0bb0b9</t>
+        </is>
+      </c>
+      <c r="P12" s="6" t="inlineStr"/>
+      <c r="Q12" s="6" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="R12" s="6" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="40" customHeight="1">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>BUG-012</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>DEFAULT_SUMMITSLIST パス誤設定（DATA_DIR/ref/ → プロジェクト直下）</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>merge.py の DEFAULT_SUMMITSLIST が DATA_DIR 配下の ref/ を参照していた。DATA_DIR は環境依存パスのためプロジェクト同梱の summitslist.csv が見つからなかった。</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>JJ1XGO</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>merge.py</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>scripts/merge.py</t>
+        </is>
+      </c>
+      <c r="I13" s="6" t="inlineStr">
+        <is>
+          <t>毎回</t>
+        </is>
+      </c>
+      <c r="J13" s="5" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="K13" s="6" t="inlineStr">
+        <is>
+          <t>解決済</t>
+        </is>
+      </c>
+      <c r="L13" s="6" t="inlineStr">
+        <is>
+          <t>JJ1XGO</t>
+        </is>
+      </c>
+      <c r="M13" s="6" t="inlineStr">
+        <is>
+          <t>COD</t>
+        </is>
+      </c>
+      <c r="N13" s="6" t="inlineStr">
+        <is>
+          <t>scripts/merge.py</t>
+        </is>
+      </c>
+      <c r="O13" s="6" t="inlineStr">
+        <is>
+          <t>Path(__file__).parent.parent / 'ref/summitslist.csv' に修正。</t>
+        </is>
+      </c>
+      <c r="P13" s="6" t="inlineStr"/>
+      <c r="Q13" s="6" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="R13" s="6" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="40" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>BUG-013</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>analyze.c: malloc(AnalyzeResult) / malloc(peaks) 後の NULL チェック漏れ</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>analyze_tile_data() 内の malloc(sizeof(AnalyzeResult)) と malloc(sizeof(PeakResult)*cnt) の後に NULL チェックがない（line 153-154）。メモリ枯渇時にヌルポインタアクセスでクラッシュする可能性がある。</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>JJ1XGO</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>COD</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>解析エンジン</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>src/analyze.c</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>まれ</t>
+        </is>
+      </c>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>未対応</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>JJ1XGO</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>COD</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>src/analyze.c</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>malloc 後に if (!result) return NULL; / if (!result-&gt;peaks) { free(result); return NULL; } を追加。</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr"/>
+      <c r="Q14" s="2" t="inlineStr"/>
+      <c r="R14" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <dataValidations count="4">
-    <dataValidation sqref="K2:K7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K2:K14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"未対応,対応中,対応完了,解決済,却下"</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"高,中,低"</formula1>
     </dataValidation>
-    <dataValidation sqref="F2:F7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"URD,SRS,HLD,LLD,COD,UT,IT,ST,OPS"</formula1>
     </dataValidation>
-    <dataValidation sqref="M2:M7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="M2:M14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"URD,SRS,HLD,LLD,COD,UT,IT,ST,OPS"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1359,214 +1975,214 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>KPI</t>
         </is>
       </c>
-      <c r="B1" s="8" t="n"/>
+      <c r="B1" s="9" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="9" t="inlineStr">
+      <c r="A2" s="10" t="inlineStr">
         <is>
           <t>合計件数</t>
         </is>
       </c>
-      <c r="B2" s="10" t="n">
+      <c r="B2" s="11" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="10" t="inlineStr">
+        <is>
+          <t>未解決件数</t>
+        </is>
+      </c>
+      <c r="B3" s="11" t="n">
         <v>6</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="9" t="inlineStr">
-        <is>
-          <t>未解決件数</t>
-        </is>
-      </c>
-      <c r="B3" s="10" t="n">
+    <row r="4">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>解決済件数</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>解決率</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>46.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>ステータス別</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>未対応</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>対応中</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>対応完了</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>解決済</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>却下</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>重大度別（未解決）</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="B17" s="11" t="n">
         <v>5</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="9" t="inlineStr">
-        <is>
-          <t>解決済件数</t>
-        </is>
-      </c>
-      <c r="B4" s="10" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="9" t="inlineStr">
-        <is>
-          <t>解決率</t>
-        </is>
-      </c>
-      <c r="B5" s="10" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>ステータス別</t>
-        </is>
-      </c>
-      <c r="B7" s="8" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="9" t="inlineStr">
-        <is>
-          <t>未対応</t>
-        </is>
-      </c>
-      <c r="B8" s="10" t="n">
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>カテゴリ別（未解決）</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>解析エンジン</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="10" t="inlineStr">
+        <is>
+          <t>merge.py</t>
+        </is>
+      </c>
+      <c r="B21" s="11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t>prefetch</t>
+        </is>
+      </c>
+      <c r="B22" s="11" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>発生源ステージ別（未解決）</t>
+        </is>
+      </c>
+      <c r="B24" s="9" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="10" t="inlineStr">
+        <is>
+          <t>COD</t>
+        </is>
+      </c>
+      <c r="B25" s="11" t="n">
         <v>5</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="9" t="inlineStr">
-        <is>
-          <t>対応中</t>
-        </is>
-      </c>
-      <c r="B9" s="10" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="9" t="inlineStr">
-        <is>
-          <t>対応完了</t>
-        </is>
-      </c>
-      <c r="B10" s="10" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="9" t="inlineStr">
-        <is>
-          <t>解決済</t>
-        </is>
-      </c>
-      <c r="B11" s="10" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="9" t="inlineStr">
-        <is>
-          <t>却下</t>
-        </is>
-      </c>
-      <c r="B12" s="10" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="7" t="inlineStr">
-        <is>
-          <t>重大度別（未解決）</t>
-        </is>
-      </c>
-      <c r="B14" s="8" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="9" t="inlineStr">
-        <is>
-          <t>高</t>
-        </is>
-      </c>
-      <c r="B15" s="10" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="9" t="inlineStr">
-        <is>
-          <t>中</t>
-        </is>
-      </c>
-      <c r="B16" s="10" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="9" t="inlineStr">
-        <is>
-          <t>低</t>
-        </is>
-      </c>
-      <c r="B17" s="10" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="7" t="inlineStr">
-        <is>
-          <t>カテゴリ別（未解決）</t>
-        </is>
-      </c>
-      <c r="B19" s="8" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="9" t="inlineStr">
-        <is>
-          <t>解析エンジン</t>
-        </is>
-      </c>
-      <c r="B20" s="10" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="9" t="inlineStr">
-        <is>
-          <t>merge.py</t>
-        </is>
-      </c>
-      <c r="B21" s="10" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="9" t="inlineStr">
-        <is>
-          <t>prefetch</t>
-        </is>
-      </c>
-      <c r="B22" s="10" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="7" t="inlineStr">
-        <is>
-          <t>発生源ステージ別（未解決）</t>
-        </is>
-      </c>
-      <c r="B24" s="8" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="9" t="inlineStr">
-        <is>
-          <t>COD</t>
-        </is>
-      </c>
-      <c r="B25" s="10" t="n">
-        <v>4</v>
-      </c>
-    </row>
     <row r="26">
-      <c r="A26" s="9" t="inlineStr">
+      <c r="A26" s="10" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="B26" s="10" t="n">
+      <c r="B26" s="11" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1581,7 +2197,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1613,8 +2229,8 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="11" t="n">
-        <v>46137</v>
+      <c r="A2" s="12" t="n">
+        <v>46130</v>
       </c>
       <c r="B2" t="n">
         <v>1</v>
@@ -1627,31 +2243,129 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="11" t="n">
+      <c r="A3" s="12" t="n">
+        <v>46131</v>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="12" t="n">
+        <v>46132</v>
+      </c>
+      <c r="B4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="n">
+        <v>46133</v>
+      </c>
+      <c r="B5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="12" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="12" t="n">
+        <v>46135</v>
+      </c>
+      <c r="B7" t="n">
+        <v>2</v>
+      </c>
+      <c r="C7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="n">
+        <v>46136</v>
+      </c>
+      <c r="B8" t="n">
+        <v>4</v>
+      </c>
+      <c r="C8" t="n">
+        <v>4</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C9" t="n">
+        <v>6</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="n">
         <v>46138</v>
       </c>
-      <c r="B3" t="n">
-        <v>6</v>
-      </c>
-      <c r="C3" t="n">
+      <c r="B10" t="n">
+        <v>12</v>
+      </c>
+      <c r="C10" t="n">
+        <v>7</v>
+      </c>
+      <c r="D10" t="n">
         <v>1</v>
       </c>
-      <c r="D3" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="11" t="n">
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="n">
         <v>46139</v>
       </c>
-      <c r="B4" t="n">
-        <v>6</v>
-      </c>
-      <c r="C4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D4" t="n">
-        <v>1</v>
+      <c r="B11" t="n">
+        <v>13</v>
+      </c>
+      <c r="C11" t="n">
+        <v>7</v>
+      </c>
+      <c r="D11" t="n">
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>